<commit_message>
Reframe D2 Fig 15 channel risk profile
</commit_message>
<xml_diff>
--- a/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/validation/D2_scientific_validation_source_data.xlsx
+++ b/Project 1 Data Quality Assessment/D2 Temporal Continuity & Information Availability/artifacts/validation/D2_scientific_validation_source_data.xlsx
@@ -24,7 +24,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="raw_vs_score_impact" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="low_tail_events" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="veto_reasons" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sensitive_diagnostics" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channel_outcome" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channel_veto" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="sensitive_diagnostics" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25791,15 +25793,914 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>display_order</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>sensor_id</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>analyte</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>n_sensor_hours</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>mean_D2_Strict</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>p05_D2_Strict</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>q25_D2_Strict</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>median_D2_Strict</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>q75_D2_Strict</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>p95_D2_Strict</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>low_hours_per_1000h</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>veto_hours_per_1000h</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>grade_A_pct</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>grade_B_pct</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>grade_C_pct</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>grade_D_pct</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>grade_E_pct</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E2" t="n">
+        <v>4.95969311097208</v>
+      </c>
+      <c r="F2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K2" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L2" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M2" t="n">
+        <v>98.02319882372161</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0.9965691880411697</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E3" t="n">
+        <v>4.959678129827932</v>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J3" t="n">
+        <v>5</v>
+      </c>
+      <c r="K3" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L3" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M3" t="n">
+        <v>98.02319882372161</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.9965691880411697</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4.959584550737319</v>
+      </c>
+      <c r="F4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G4" t="n">
+        <v>5</v>
+      </c>
+      <c r="H4" t="n">
+        <v>5</v>
+      </c>
+      <c r="I4" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" t="n">
+        <v>5</v>
+      </c>
+      <c r="K4" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L4" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M4" t="n">
+        <v>98.03953602352557</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0.9802319882372161</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ORP_1_2</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E5" t="n">
+        <v>4.959549489076767</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" t="n">
+        <v>5</v>
+      </c>
+      <c r="H5" t="n">
+        <v>5</v>
+      </c>
+      <c r="I5" t="n">
+        <v>5</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L5" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M5" t="n">
+        <v>98.03953602352557</v>
+      </c>
+      <c r="N5" t="n">
+        <v>0.9802319882372161</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E6" t="n">
+        <v>4.959297978162197</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5</v>
+      </c>
+      <c r="I6" t="n">
+        <v>5</v>
+      </c>
+      <c r="J6" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L6" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M6" t="n">
+        <v>98.03953602352557</v>
+      </c>
+      <c r="N6" t="n">
+        <v>0.9802319882372161</v>
+      </c>
+      <c r="O6" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ORP_2_3</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E7" t="n">
+        <v>4.958891111258255</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" t="n">
+        <v>5</v>
+      </c>
+      <c r="K7" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L7" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M7" t="n">
+        <v>98.02319882372161</v>
+      </c>
+      <c r="N7" t="n">
+        <v>0.9965691880411697</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DO_1_2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E8" t="n">
+        <v>4.958802624313989</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" t="n">
+        <v>5</v>
+      </c>
+      <c r="I8" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" t="n">
+        <v>5</v>
+      </c>
+      <c r="K8" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L8" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M8" t="n">
+        <v>97.94151282470185</v>
+      </c>
+      <c r="N8" t="n">
+        <v>1.078255187060938</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DO_1_1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E9" t="n">
+        <v>4.958750182170779</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I9" t="n">
+        <v>5</v>
+      </c>
+      <c r="J9" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L9" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M9" t="n">
+        <v>97.94151282470185</v>
+      </c>
+      <c r="N9" t="n">
+        <v>1.078255187060938</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DO_1_3</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4.958655165394208</v>
+      </c>
+      <c r="F10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J10" t="n">
+        <v>5</v>
+      </c>
+      <c r="K10" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L10" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M10" t="n">
+        <v>97.94151282470185</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1.078255187060938</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>DO_1_4</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4.958468053604856</v>
+      </c>
+      <c r="F11" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
+      <c r="I11" t="n">
+        <v>5</v>
+      </c>
+      <c r="J11" t="n">
+        <v>5</v>
+      </c>
+      <c r="K11" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="L11" t="n">
+        <v>9.312203888253554</v>
+      </c>
+      <c r="M11" t="n">
+        <v>97.94151282470185</v>
+      </c>
+      <c r="N11" t="n">
+        <v>1.078255187060938</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.04901159941186081</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>DO_2_3</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4.950962435055505</v>
+      </c>
+      <c r="F12" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" t="n">
+        <v>5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>12.41627185100474</v>
+      </c>
+      <c r="L12" t="n">
+        <v>12.41627185100474</v>
+      </c>
+      <c r="M12" t="n">
+        <v>97.64744322823069</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1.045580787453031</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.3757555954909328</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>DO_2_2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E13" t="n">
+        <v>4.950919242267472</v>
+      </c>
+      <c r="F13" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>5</v>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>12.41627185100474</v>
+      </c>
+      <c r="L13" t="n">
+        <v>12.41627185100474</v>
+      </c>
+      <c r="M13" t="n">
+        <v>97.64744322823069</v>
+      </c>
+      <c r="N13" t="n">
+        <v>1.045580787453031</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.3757555954909328</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DO_2_4</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4.950880157238672</v>
+      </c>
+      <c r="F14" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" t="n">
+        <v>5</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5</v>
+      </c>
+      <c r="J14" t="n">
+        <v>5</v>
+      </c>
+      <c r="K14" t="n">
+        <v>12.41627185100474</v>
+      </c>
+      <c r="L14" t="n">
+        <v>12.41627185100474</v>
+      </c>
+      <c r="M14" t="n">
+        <v>97.64744322823069</v>
+      </c>
+      <c r="N14" t="n">
+        <v>1.045580787453031</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0.3757555954909328</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>DO_2_1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>6121</v>
+      </c>
+      <c r="E15" t="n">
+        <v>4.940616378333655</v>
+      </c>
+      <c r="F15" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+      <c r="H15" t="n">
+        <v>5</v>
+      </c>
+      <c r="I15" t="n">
+        <v>5</v>
+      </c>
+      <c r="J15" t="n">
+        <v>5</v>
+      </c>
+      <c r="K15" t="n">
+        <v>12.57964384904427</v>
+      </c>
+      <c r="L15" t="n">
+        <v>12.57964384904427</v>
+      </c>
+      <c r="M15" t="n">
+        <v>96.61819964058161</v>
+      </c>
+      <c r="N15" t="n">
+        <v>2.009475575886293</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.4411043947067473</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0.9312203888253554</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sensor_id</t>
+        </is>
+      </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>analyte</t>
@@ -25807,273 +26708,260 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>soft_stasis_fraction</t>
+          <t>reason_group</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>intrinsic_soft_hour_rate</t>
+          <t>veto_hours</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>peer_response_loss_hour_rate</t>
+          <t>veto_share_pct</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>joint_soft_hour_rate</t>
+          <t>veto_hours_per_1000h</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>sustained_quasi_freeze_hour_rate</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>production_Q_HA_low_rate</t>
+          <t>display_order</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>DO_1_1</t>
+          <t>ORP_2_1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>0.002295376572455481</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="E2" t="n">
-        <v>0.008495343898055873</v>
+        <v>43.85964912280701</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>4.084299950988401</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>DO_1_2</t>
+          <t>ORP_2_1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>0.0007787398573217884</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0040842999509884</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>0.490115994118608</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DO_1_3</t>
+          <t>ORP_2_1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>0.0009257746555573707</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01306975984316288</v>
+        <v>50.87719298245614</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>4.737787943146545</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DO_1_4</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>0.5849479932472906</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
       </c>
       <c r="D5" t="n">
-        <v>0.7026629635680445</v>
+        <v>25</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
+        <v>43.85964912280701</v>
       </c>
       <c r="F5" t="n">
-        <v>0</v>
+        <v>4.084299950988401</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>DO_2_1</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C6" t="n">
-        <v>0.02782724318829531</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
       </c>
       <c r="D6" t="n">
-        <v>0.01437673582747917</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n">
-        <v>0.01176278385884659</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="F6" t="n">
-        <v>0.002613951968632576</v>
+        <v>0.490115994118608</v>
       </c>
       <c r="G6" t="n">
-        <v>0.001960463976474432</v>
-      </c>
-      <c r="H6" t="n">
-        <v>0.00571801993138376</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DO_2_2</t>
+          <t>ORP_2_2</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>0.006793552251810706</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
       </c>
       <c r="D7" t="n">
-        <v>0.003104067962751185</v>
+        <v>29</v>
       </c>
       <c r="E7" t="n">
-        <v>0.03528835157653978</v>
+        <v>50.87719298245614</v>
       </c>
       <c r="F7" t="n">
-        <v>0.001960463976474432</v>
+        <v>4.737787943146545</v>
       </c>
       <c r="G7" t="n">
-        <v>0.001470347982355824</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.003594183956869793</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DO_2_3</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>0.003076839296411261</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
       </c>
       <c r="D8" t="n">
-        <v>0.003104067962751185</v>
+        <v>25</v>
       </c>
       <c r="E8" t="n">
-        <v>0.000163371998039536</v>
+        <v>43.85964912280701</v>
       </c>
       <c r="F8" t="n">
-        <v>0.000163371998039536</v>
+        <v>4.084299950988401</v>
       </c>
       <c r="G8" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.003594183956869793</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DO_2_4</t>
+          <t>ORP_1_1</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>DO</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>0.1935967252990615</v>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
       </c>
       <c r="D9" t="n">
-        <v>0.1385394543375265</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>0.490115994118608</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.003594183956869793</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -26087,23 +26975,22 @@
           <t>ORP</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>0.1203293761004919</v>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
       </c>
       <c r="D10" t="n">
-        <v>0.002123835974513968</v>
+        <v>29</v>
       </c>
       <c r="E10" t="n">
-        <v>0.01911452377062571</v>
+        <v>50.87719298245614</v>
       </c>
       <c r="F10" t="n">
-        <v>0.000490115994118608</v>
+        <v>4.737787943146545</v>
       </c>
       <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -26117,29 +27004,28 @@
           <t>ORP</t>
         </is>
       </c>
-      <c r="C11" t="n">
-        <v>0.116784203743034</v>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
       </c>
       <c r="D11" t="n">
-        <v>0.01143603986276752</v>
+        <v>25</v>
       </c>
       <c r="E11" t="n">
-        <v>0.009148831890214017</v>
+        <v>43.85964912280701</v>
       </c>
       <c r="F11" t="n">
-        <v>0.00163371998039536</v>
+        <v>4.084299950988401</v>
       </c>
       <c r="G11" t="n">
-        <v>0.000326743996079072</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ORP_1_3</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -26147,29 +27033,28 @@
           <t>ORP</t>
         </is>
       </c>
-      <c r="C12" t="n">
-        <v>0.09343607616765598</v>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
       </c>
       <c r="D12" t="n">
-        <v>0.07319065512171213</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0.01012906387845123</v>
+        <v>5.263157894736842</v>
       </c>
       <c r="F12" t="n">
-        <v>0.009148831890214017</v>
+        <v>0.490115994118608</v>
       </c>
       <c r="G12" t="n">
-        <v>0.005391275935304689</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ORP_2_1</t>
+          <t>ORP_1_2</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -26177,29 +27062,28 @@
           <t>ORP</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>0.2089064967597887</v>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
       </c>
       <c r="D13" t="n">
-        <v>0.04378369547459565</v>
+        <v>29</v>
       </c>
       <c r="E13" t="n">
-        <v>0.02908021565103741</v>
+        <v>50.87719298245614</v>
       </c>
       <c r="F13" t="n">
-        <v>0.009148831890214017</v>
+        <v>4.737787943146545</v>
       </c>
       <c r="G13" t="n">
-        <v>0.00163371998039536</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ORP_2_2</t>
+          <t>ORP_1_3</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -26207,53 +27091,979 @@
           <t>ORP</t>
         </is>
       </c>
-      <c r="C14" t="n">
-        <v>0.379582584545009</v>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
       </c>
       <c r="D14" t="n">
-        <v>0.2707074007515112</v>
+        <v>25</v>
       </c>
       <c r="E14" t="n">
-        <v>0.1079888907041333</v>
+        <v>43.85964912280701</v>
       </c>
       <c r="F14" t="n">
-        <v>0.08201274301584709</v>
+        <v>4.084299950988401</v>
       </c>
       <c r="G14" t="n">
-        <v>0.04247671949027937</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G15" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>29</v>
+      </c>
+      <c r="E16" t="n">
+        <v>50.87719298245614</v>
+      </c>
+      <c r="F16" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G16" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>ORP_2_3</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>ORP</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>0.3069455789722086</v>
-      </c>
-      <c r="D15" t="n">
-        <v>0.3051788923378533</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.1414801503022382</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0.1351086423786963</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0.1003104067962751</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0</v>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>25</v>
+      </c>
+      <c r="E17" t="n">
+        <v>43.85964912280701</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ORP_2_3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="F18" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ORP_2_3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>29</v>
+      </c>
+      <c r="E19" t="n">
+        <v>50.87719298245614</v>
+      </c>
+      <c r="F19" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G19" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>DO_1_2</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>25</v>
+      </c>
+      <c r="E20" t="n">
+        <v>43.85964912280701</v>
+      </c>
+      <c r="F20" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G20" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>DO_1_2</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="F21" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G21" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>DO_1_2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>29</v>
+      </c>
+      <c r="E22" t="n">
+        <v>50.87719298245614</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G22" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>DO_1_1</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>25</v>
+      </c>
+      <c r="E23" t="n">
+        <v>43.85964912280701</v>
+      </c>
+      <c r="F23" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G23" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>DO_1_1</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G24" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>DO_1_1</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>29</v>
+      </c>
+      <c r="E25" t="n">
+        <v>50.87719298245614</v>
+      </c>
+      <c r="F25" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G25" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>DO_1_3</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>25</v>
+      </c>
+      <c r="E26" t="n">
+        <v>43.85964912280701</v>
+      </c>
+      <c r="F26" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G26" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>DO_1_3</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G27" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>DO_1_3</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>29</v>
+      </c>
+      <c r="E28" t="n">
+        <v>50.87719298245614</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G28" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DO_1_4</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>25</v>
+      </c>
+      <c r="E29" t="n">
+        <v>43.85964912280701</v>
+      </c>
+      <c r="F29" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G29" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DO_1_4</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3</v>
+      </c>
+      <c r="E30" t="n">
+        <v>5.263157894736842</v>
+      </c>
+      <c r="F30" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G30" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DO_1_4</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>29</v>
+      </c>
+      <c r="E31" t="n">
+        <v>50.87719298245614</v>
+      </c>
+      <c r="F31" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G31" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DO_2_3</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>25</v>
+      </c>
+      <c r="E32" t="n">
+        <v>32.89473684210527</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G32" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DO_2_3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" t="n">
+        <v>3.947368421052631</v>
+      </c>
+      <c r="F33" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G33" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DO_2_3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Hard stasis</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>19</v>
+      </c>
+      <c r="E34" t="n">
+        <v>25</v>
+      </c>
+      <c r="F34" t="n">
+        <v>3.104067962751185</v>
+      </c>
+      <c r="G34" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DO_2_3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>29</v>
+      </c>
+      <c r="E35" t="n">
+        <v>38.15789473684211</v>
+      </c>
+      <c r="F35" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G35" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DO_2_2</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>25</v>
+      </c>
+      <c r="E36" t="n">
+        <v>32.89473684210527</v>
+      </c>
+      <c r="F36" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G36" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>DO_2_2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>3</v>
+      </c>
+      <c r="E37" t="n">
+        <v>3.947368421052631</v>
+      </c>
+      <c r="F37" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G37" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>DO_2_2</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Hard stasis</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>19</v>
+      </c>
+      <c r="E38" t="n">
+        <v>25</v>
+      </c>
+      <c r="F38" t="n">
+        <v>3.104067962751185</v>
+      </c>
+      <c r="G38" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DO_2_2</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>29</v>
+      </c>
+      <c r="E39" t="n">
+        <v>38.15789473684211</v>
+      </c>
+      <c r="F39" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G39" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DO_2_4</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>25</v>
+      </c>
+      <c r="E40" t="n">
+        <v>32.89473684210527</v>
+      </c>
+      <c r="F40" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G40" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>DO_2_4</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>3</v>
+      </c>
+      <c r="E41" t="n">
+        <v>3.947368421052631</v>
+      </c>
+      <c r="F41" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G41" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DO_2_4</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Hard stasis</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>19</v>
+      </c>
+      <c r="E42" t="n">
+        <v>25</v>
+      </c>
+      <c r="F42" t="n">
+        <v>3.104067962751185</v>
+      </c>
+      <c r="G42" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>DO_2_4</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>29</v>
+      </c>
+      <c r="E43" t="n">
+        <v>38.15789473684211</v>
+      </c>
+      <c r="F43" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G43" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>DO_2_1</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Gap + missing</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>25</v>
+      </c>
+      <c r="E44" t="n">
+        <v>32.46753246753246</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4.084299950988401</v>
+      </c>
+      <c r="G44" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>DO_2_1</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Gap only</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>3</v>
+      </c>
+      <c r="E45" t="n">
+        <v>3.896103896103896</v>
+      </c>
+      <c r="F45" t="n">
+        <v>0.490115994118608</v>
+      </c>
+      <c r="G45" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>DO_2_1</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Hard stasis</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>20</v>
+      </c>
+      <c r="E46" t="n">
+        <v>25.97402597402597</v>
+      </c>
+      <c r="F46" t="n">
+        <v>3.26743996079072</v>
+      </c>
+      <c r="G46" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>DO_2_1</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Missing only</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>29</v>
+      </c>
+      <c r="E47" t="n">
+        <v>37.66233766233766</v>
+      </c>
+      <c r="F47" t="n">
+        <v>4.737787943146545</v>
+      </c>
+      <c r="G47" t="n">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -26609,6 +28419,482 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>sensor_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>analyte</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>soft_stasis_fraction</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>intrinsic_soft_hour_rate</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>peer_response_loss_hour_rate</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>joint_soft_hour_rate</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>sustained_quasi_freeze_hour_rate</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>production_Q_HA_low_rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DO_1_1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>0.002295376572455481</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.008495343898055873</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DO_1_2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>0.0007787398573217884</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0040842999509884</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DO_1_3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.0009257746555573707</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.01306975984316288</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DO_1_4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>0.5849479932472906</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.7026629635680445</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DO_2_1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.02782724318829531</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.01437673582747917</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.01176278385884659</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.002613951968632576</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.001960463976474432</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.00571801993138376</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DO_2_2</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.006793552251810706</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.003104067962751185</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.03528835157653978</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.001960463976474432</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.001470347982355824</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.003594183956869793</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DO_2_3</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>0.003076839296411261</v>
+      </c>
+      <c r="D8" t="n">
+        <v>0.003104067962751185</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0.000163371998039536</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.000163371998039536</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.003594183956869793</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DO_2_4</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DO</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.1935967252990615</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.1385394543375265</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.003594183956869793</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ORP_1_1</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.1203293761004919</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.002123835974513968</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.01911452377062571</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.000490115994118608</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ORP_1_2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>0.116784203743034</v>
+      </c>
+      <c r="D11" t="n">
+        <v>0.01143603986276752</v>
+      </c>
+      <c r="E11" t="n">
+        <v>0.009148831890214017</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.00163371998039536</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.000326743996079072</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ORP_1_3</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>0.09343607616765598</v>
+      </c>
+      <c r="D12" t="n">
+        <v>0.07319065512171213</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0.01012906387845123</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0.009148831890214017</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.005391275935304689</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORP_2_1</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>0.2089064967597887</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.04378369547459565</v>
+      </c>
+      <c r="E13" t="n">
+        <v>0.02908021565103741</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.009148831890214017</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.00163371998039536</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORP_2_2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0.379582584545009</v>
+      </c>
+      <c r="D14" t="n">
+        <v>0.2707074007515112</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0.1079888907041333</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0.08201274301584709</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.04247671949027937</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ORP_2_3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ORP</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0.3069455789722086</v>
+      </c>
+      <c r="D15" t="n">
+        <v>0.3051788923378533</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0.1414801503022382</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0.1351086423786963</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.1003104067962751</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>